<commit_message>
An intermediate commit, several thing have been updated => (1) Fission Detector in PoP infile (2) gen_events to launch classic GEFbashscript.sh (3) event_generator.py fixed for light and heavy (2*eventID-1 for light and 2*eventID for heavy) to be simulated later  (4) FissioHistoTest.cpp to check if everything worked (5) Fragment and Fission event class in det_analysis
</commit_message>
<xml_diff>
--- a/ReacInfoFiles/Qi_dipole-old_ESR_std.xlsx
+++ b/ReacInfoFiles/Qi_dipole-old_ESR_std.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\G4bl_simulations\NECTAR_G4bl_Sim\Code\ReacInfoFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\Simulation\NECTAR_G4bl_Simulation\ReacInfoFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5588549-A368-4E21-8BA3-1B90230D6B45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294C8AC7-B55C-471D-AF94-704B04CE550A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="3075" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GPAC" sheetId="7" r:id="rId1"/>
@@ -452,9 +452,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -492,7 +492,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -598,7 +598,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -740,7 +740,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -774,7 +774,7 @@
         <v>19</v>
       </c>
       <c r="B6">
-        <v>238.05078783332203</v>
+        <v>238.05078825999999</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -791,7 +791,7 @@
       </c>
       <c r="B8" s="4">
         <f>SQRT((B7*B6+B6*931.5)^2-(931.5*B6)^2)</f>
-        <v>42859.282631582784</v>
+        <v>42859.282708402869</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -800,7 +800,7 @@
       </c>
       <c r="B9" s="4">
         <f>$B$8/(2.997925*100*$B$5)</f>
-        <v>1.5539473727147792</v>
+        <v>1.5539473755000419</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -817,7 +817,7 @@
       </c>
       <c r="B11" s="6">
         <f>B9/B10</f>
-        <v>0.24444665293609866</v>
+        <v>0.24444665337423971</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -925,7 +925,7 @@
       </c>
       <c r="B26" s="21">
         <f>B14*B19*$B$9</f>
-        <v>-0.79325257797079107</v>
+        <v>-0.7932525793926003</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -934,7 +934,7 @@
       </c>
       <c r="B27" s="22">
         <f>B15*B20*$B$9</f>
-        <v>0.71411311198633054</v>
+        <v>0.7141131132662919</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -943,7 +943,7 @@
       </c>
       <c r="B28" s="22">
         <f>B16*B21*$B$9</f>
-        <v>0.5233738355066655</v>
+        <v>0.52337383644474977</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
@@ -952,7 +952,7 @@
       </c>
       <c r="B29" s="22">
         <f>B17*B22*$B$9</f>
-        <v>-0.70769936669360867</v>
+        <v>-0.70769936796207422</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -961,7 +961,7 @@
       </c>
       <c r="B30" s="23">
         <f>B18*B23*$B$9</f>
-        <v>0.65463988804042061</v>
+        <v>0.65463988921378335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>